<commit_message>
Clarify Target R semantics: applicable target type, R sign shows hit vs stopped out
</commit_message>
<xml_diff>
--- a/templates/trade_enrichment_template.xlsx
+++ b/templates/trade_enrichment_template.xlsx
@@ -239,17 +239,17 @@
     </comment>
     <comment ref="N1" authorId="0" shapeId="0">
       <text>
-        <t>R achieved if the target was the nearest Classic Level. Use negative values for losses (e.g. -1). Leave blank if this target type wasn't used.</t>
+        <t>R outcome when the nearest Classic Level was the applicable target for this trade. Positive = target hit, negative = stopped out first (e.g. -1 for a 1R loss). Leave blank if this target type didn't apply to this trade.</t>
       </text>
     </comment>
     <comment ref="O1" authorId="0" shapeId="0">
       <text>
-        <t>R achieved if the target was a further recent S/R zone. Leave blank if this target type wasn't used.</t>
+        <t>R outcome when a further recent S/R zone was the applicable target. Positive = target hit, negative = stopped out first (e.g. -1). Leave blank if this target type didn't apply to this trade.</t>
       </text>
     </comment>
     <comment ref="P1" authorId="0" shapeId="0">
       <text>
-        <t>R achieved if the target was the IB high/low. Leave blank if this target type wasn't used.</t>
+        <t>R outcome when the IB high/low was the applicable target. Positive = target hit, negative = stopped out first (e.g. -1). Leave blank if this target type didn't apply to this trade.</t>
       </text>
     </comment>
     <comment ref="Q1" authorId="0" shapeId="0">

</xml_diff>

<commit_message>
Add entryBasis field: categorical reason for entry (support/resistance/classic_level/confluence)
</commit_message>
<xml_diff>
--- a/templates/trade_enrichment_template.xlsx
+++ b/templates/trade_enrichment_template.xlsx
@@ -204,70 +204,75 @@
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
+        <t>The categorical reason this entry was taken: a support zone, a resistance zone, a classic level alone, or a zone + classic level confluence.</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
         <t>Lower boundary price of the S/R zone this trade was based on.</t>
       </text>
     </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
+    <comment ref="I1" authorId="0" shapeId="0">
       <text>
         <t>Upper boundary price of the S/R zone this trade was based on.</t>
       </text>
     </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
+    <comment ref="J1" authorId="0" shapeId="0">
       <text>
         <t>Classic Level price used as target reference, if applicable.</t>
       </text>
     </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
+    <comment ref="K1" authorId="0" shapeId="0">
       <text>
         <t>Whether the zone acted as support or resistance for this trade.</t>
       </text>
     </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
+    <comment ref="L1" authorId="0" shapeId="0">
       <text>
         <t>Number of times price touched/respected this zone before this trade.</t>
       </text>
     </comment>
-    <comment ref="L1" authorId="0" shapeId="0">
+    <comment ref="M1" authorId="0" shapeId="0">
       <text>
         <t>Number of times price broke through this zone before this trade.</t>
       </text>
     </comment>
-    <comment ref="M1" authorId="0" shapeId="0">
+    <comment ref="N1" authorId="0" shapeId="0">
       <text>
         <t>Where the stop loss was placed for this trade.</t>
       </text>
     </comment>
-    <comment ref="N1" authorId="0" shapeId="0">
+    <comment ref="O1" authorId="0" shapeId="0">
       <text>
         <t>R outcome when the nearest Classic Level was the applicable target for this trade. Positive = target hit, negative = stopped out first (e.g. -1 for a 1R loss). Leave blank if this target type didn't apply to this trade.</t>
       </text>
     </comment>
-    <comment ref="O1" authorId="0" shapeId="0">
+    <comment ref="P1" authorId="0" shapeId="0">
       <text>
         <t>R outcome when a further recent S/R zone was the applicable target. Positive = target hit, negative = stopped out first (e.g. -1). Leave blank if this target type didn't apply to this trade.</t>
       </text>
     </comment>
-    <comment ref="P1" authorId="0" shapeId="0">
+    <comment ref="Q1" authorId="0" shapeId="0">
       <text>
         <t>R outcome when the IB high/low was the applicable target. Positive = target hit, negative = stopped out first (e.g. -1). Leave blank if this target type didn't apply to this trade.</t>
       </text>
     </comment>
-    <comment ref="Q1" authorId="0" shapeId="0">
+    <comment ref="R1" authorId="0" shapeId="0">
       <text>
         <t>R achieved with default management: fixed SL, no trailing (your actual executed outcome in most trades).</t>
       </text>
     </comment>
-    <comment ref="R1" authorId="0" shapeId="0">
+    <comment ref="S1" authorId="0" shapeId="0">
       <text>
         <t>Hypothetical/actual R if target was extended further without moving SL. Fill only if you evaluated this alternative on this trade.</t>
       </text>
     </comment>
-    <comment ref="S1" authorId="0" shapeId="0">
+    <comment ref="T1" authorId="0" shapeId="0">
       <text>
         <t>Hypothetical/actual R if 50% was booked and SL trailed to swing high/low, letting the rest run. Fill only if evaluated on this trade.</t>
       </text>
     </comment>
-    <comment ref="T1" authorId="0" shapeId="0">
+    <comment ref="U1" authorId="0" shapeId="0">
       <text>
         <t>Free-text observations, mistakes, rationale for this trade.</t>
       </text>
@@ -565,7 +570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T2"/>
+  <dimension ref="A1:U2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -581,13 +586,14 @@
     <col width="18" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
     <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="23" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="23" customWidth="1" min="15" max="15"/>
     <col width="20" customWidth="1" min="16" max="16"/>
-    <col width="18" customWidth="1" min="17" max="17"/>
-    <col width="23" customWidth="1" min="18" max="18"/>
-    <col width="25" customWidth="1" min="19" max="19"/>
-    <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="23" customWidth="1" min="19" max="19"/>
+    <col width="25" customWidth="1" min="20" max="20"/>
+    <col width="18" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -623,70 +629,75 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>entryBasis</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>srZoneLow</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>srZoneHigh</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>classicLevel</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>srType</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>srTouchCount</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>srFailureCount</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>slPlacement</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>targetClassicLevelR</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>targetFurtherSrR</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>targetIbHighLowR</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>mgmtNoMoveR</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>mgmtExtendedTargetR</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>mgmtPartialBookTrailR</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -723,26 +734,26 @@
           <t>(text)</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>(text)</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>(number)</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>(number)</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>(number)</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>(text)</t>
-        </is>
-      </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
           <t>(text)</t>
@@ -758,44 +769,49 @@
           <t>(text)</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>(text)</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr">
         <is>
           <t>(number)</t>
         </is>
       </c>
-      <c r="O2" s="3" t="inlineStr">
+      <c r="P2" s="3" t="inlineStr">
         <is>
           <t>(number)</t>
         </is>
       </c>
-      <c r="P2" s="3" t="inlineStr">
+      <c r="Q2" s="3" t="inlineStr">
         <is>
           <t>(number)</t>
         </is>
       </c>
-      <c r="Q2" s="3" t="inlineStr">
+      <c r="R2" s="3" t="inlineStr">
         <is>
           <t>(number)</t>
         </is>
       </c>
-      <c r="R2" s="3" t="inlineStr">
+      <c r="S2" s="3" t="inlineStr">
         <is>
           <t>(number)</t>
         </is>
       </c>
-      <c r="S2" s="3" t="inlineStr">
+      <c r="T2" s="3" t="inlineStr">
         <is>
           <t>(number)</t>
         </is>
       </c>
-      <c r="T2" s="2" t="inlineStr">
+      <c r="U2" s="2" t="inlineStr">
         <is>
           <t>(text)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="10">
+  <dataValidations count="11">
     <dataValidation sqref="A3:A1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Value must be one of: 01:30-02:30, 03:00-04:30, 14:00-16:00" type="list">
       <formula1>"01:30-02:30,03:00-04:30,14:00-16:00"</formula1>
     </dataValidation>
@@ -814,16 +830,19 @@
     <dataValidation sqref="F3:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Value must be one of: A, B, C" type="list">
       <formula1>"A,B,C"</formula1>
     </dataValidation>
-    <dataValidation sqref="J3:J1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Value must be one of: support, resistance" type="list">
+    <dataValidation sqref="G3:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Value must be one of: support, resistance, classic_level, support_confluence, resistance_confluence" type="list">
+      <formula1>"support,resistance,classic_level,support_confluence,resistance_confluence"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K3:K1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Value must be one of: support, resistance" type="list">
       <formula1>"support,resistance"</formula1>
     </dataValidation>
-    <dataValidation sqref="K3:K1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Value must be one of: 1, 2, 3, 4, 4+" type="list">
+    <dataValidation sqref="L3:L1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Value must be one of: 1, 2, 3, 4, 4+" type="list">
       <formula1>"1,2,3,4,4+"</formula1>
     </dataValidation>
-    <dataValidation sqref="L3:L1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Value must be one of: 0, 1, 2, 3, 4+" type="list">
+    <dataValidation sqref="M3:M1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Value must be one of: 0, 1, 2, 3, 4+" type="list">
       <formula1>"0,1,2,3,4+"</formula1>
     </dataValidation>
-    <dataValidation sqref="M3:M1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Value must be one of: above_sr, candle_high_low, swing_high_low" type="list">
+    <dataValidation sqref="N3:N1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Value must be one of: above_sr, candle_high_low, swing_high_low" type="list">
       <formula1>"above_sr,candle_high_low,swing_high_low"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>